<commit_message>
data: msg 874 recovery + 2 overnight rows (msgs 922, 924)
- msg 874 recovered: row was already in Excel from the original failed
  run (the print crash happened AFTER writer.save), but state.json had
  marked it "failed". Reprocessing via `scripts/reprocess.py --msg-id
  874 --update` confirmed the Excel row was correct (name: غالب عبد
  الرحمن أبو شاويش, birth 1974-05-22, mart 2025-11-22, rank قائد
  سرية, battalion كتيبة القدس, brigade لواء الوسطى). state.json
  manually patched to add 874 back to processed_msg_ids with status
  "complete".

- 2 overnight messages auto-fetched + processed:
  - msg 922: birth=1987-02-15, mart=2024-11-05
  - msg 924: birth=1962-01-08, mart=2023-11-29

- data/martyrs.json regenerated: 424 → 426 rows.
- data/photos/922.jpg + data/photos/924.jpg added.

state.json (gitignored): 681 processed msg_ids, range 20-924, includes
the recovered 874.
</commit_message>
<xml_diff>
--- a/data/martyrs.xlsx
+++ b/data/martyrs.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P426"/>
+  <dimension ref="A1:P428"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27044,13 +27044,11 @@
           <t>2023-11-01</t>
         </is>
       </c>
-      <c r="F391" t="inlineStr"/>
       <c r="G391" t="inlineStr">
         <is>
           <t>نائب قائد مجموعة</t>
         </is>
       </c>
-      <c r="H391" t="inlineStr"/>
       <c r="I391" t="inlineStr">
         <is>
           <t>كتيبة المدفعية</t>
@@ -27116,13 +27114,11 @@
           <t>2025-05-15</t>
         </is>
       </c>
-      <c r="F392" t="inlineStr"/>
       <c r="G392" t="inlineStr">
         <is>
           <t>مجاهد قسا مو</t>
         </is>
       </c>
-      <c r="H392" t="inlineStr"/>
       <c r="I392" t="inlineStr">
         <is>
           <t>كتيبة المدفعية</t>
@@ -27188,13 +27184,11 @@
           <t>2024-03-24</t>
         </is>
       </c>
-      <c r="F393" t="inlineStr"/>
       <c r="G393" t="inlineStr">
         <is>
           <t>مجاهد قسا مو</t>
         </is>
       </c>
-      <c r="H393" t="inlineStr"/>
       <c r="I393" t="inlineStr">
         <is>
           <t>كتيبة المدفعية</t>
@@ -27256,13 +27250,11 @@
           <t>2023-12-03</t>
         </is>
       </c>
-      <c r="F394" t="inlineStr"/>
       <c r="G394" t="inlineStr">
         <is>
           <t>قائد مجموعة</t>
         </is>
       </c>
-      <c r="H394" t="inlineStr"/>
       <c r="I394" t="inlineStr">
         <is>
           <t>كتيبة المدفعية</t>
@@ -27328,13 +27320,11 @@
           <t>2024-02-03</t>
         </is>
       </c>
-      <c r="F395" t="inlineStr"/>
       <c r="G395" t="inlineStr">
         <is>
           <t>مجاهد قسا مو</t>
         </is>
       </c>
-      <c r="H395" t="inlineStr"/>
       <c r="I395" t="inlineStr">
         <is>
           <t>كتيبة المدفعية</t>
@@ -27400,13 +27390,11 @@
           <t>2025-03-18</t>
         </is>
       </c>
-      <c r="F396" t="inlineStr"/>
       <c r="G396" t="inlineStr">
         <is>
           <t>قائدسرية</t>
         </is>
       </c>
-      <c r="H396" t="inlineStr"/>
       <c r="I396" t="inlineStr">
         <is>
           <t>كتيبة التفاح والدرج</t>
@@ -27472,13 +27460,11 @@
           <t>2023-12-15</t>
         </is>
       </c>
-      <c r="F397" t="inlineStr"/>
       <c r="G397" t="inlineStr">
         <is>
           <t>قائد مجموعة</t>
         </is>
       </c>
-      <c r="H397" t="inlineStr"/>
       <c r="I397" t="inlineStr">
         <is>
           <t>كتيبة الرضوان</t>
@@ -27544,13 +27530,11 @@
           <t>2023-12-07</t>
         </is>
       </c>
-      <c r="F398" t="inlineStr"/>
       <c r="G398" t="inlineStr">
         <is>
           <t>قائدفصيل</t>
         </is>
       </c>
-      <c r="H398" t="inlineStr"/>
       <c r="I398" t="inlineStr">
         <is>
           <t>كتيبة الشجاعية</t>
@@ -27616,13 +27600,11 @@
           <t>2023-10-29</t>
         </is>
       </c>
-      <c r="F399" t="inlineStr"/>
       <c r="G399" t="inlineStr">
         <is>
           <t>قائد فصيل</t>
         </is>
       </c>
-      <c r="H399" t="inlineStr"/>
       <c r="I399" t="inlineStr">
         <is>
           <t>كتيبة الرضوان</t>
@@ -27688,13 +27670,11 @@
           <t>2023-12-07</t>
         </is>
       </c>
-      <c r="F400" t="inlineStr"/>
       <c r="G400" t="inlineStr">
         <is>
           <t>نائب قائد كتيبة</t>
         </is>
       </c>
-      <c r="H400" t="inlineStr"/>
       <c r="I400" t="inlineStr">
         <is>
           <t>كتيبة الشجاعية</t>
@@ -27760,13 +27740,11 @@
           <t>2025-09-05</t>
         </is>
       </c>
-      <c r="F401" t="inlineStr"/>
       <c r="G401" t="inlineStr">
         <is>
           <t>قائدفصيل</t>
         </is>
       </c>
-      <c r="H401" t="inlineStr"/>
       <c r="I401" t="inlineStr">
         <is>
           <t>كتيبة الزيتون</t>
@@ -27832,13 +27810,11 @@
           <t>2024-08-03</t>
         </is>
       </c>
-      <c r="F402" t="inlineStr"/>
       <c r="G402" t="inlineStr">
         <is>
           <t>قائد فصيل</t>
         </is>
       </c>
-      <c r="H402" t="inlineStr"/>
       <c r="I402" t="inlineStr">
         <is>
           <t>كتيبة الرضوان</t>
@@ -27904,13 +27880,11 @@
           <t>29</t>
         </is>
       </c>
-      <c r="F403" t="inlineStr"/>
       <c r="G403" t="inlineStr">
         <is>
           <t>قائدسرية</t>
         </is>
       </c>
-      <c r="H403" t="inlineStr"/>
       <c r="I403" t="inlineStr">
         <is>
           <t>كتيبة التفاح والدرج</t>
@@ -27976,13 +27950,11 @@
           <t>2024-10-17</t>
         </is>
       </c>
-      <c r="F404" t="inlineStr"/>
       <c r="G404" t="inlineStr">
         <is>
           <t>قائد فصيل</t>
         </is>
       </c>
-      <c r="H404" t="inlineStr"/>
       <c r="I404" t="inlineStr">
         <is>
           <t>كتيبة حطين</t>
@@ -28048,13 +28020,11 @@
           <t>2023-12-24</t>
         </is>
       </c>
-      <c r="F405" t="inlineStr"/>
       <c r="G405" t="inlineStr">
         <is>
           <t>قائد فصيل</t>
         </is>
       </c>
-      <c r="H405" t="inlineStr"/>
       <c r="I405" t="inlineStr">
         <is>
           <t>كتيبة حطين</t>
@@ -28192,13 +28162,11 @@
           <t>2025-03-18</t>
         </is>
       </c>
-      <c r="F407" t="inlineStr"/>
       <c r="G407" t="inlineStr">
         <is>
           <t>قائد كتيبة</t>
         </is>
       </c>
-      <c r="H407" t="inlineStr"/>
       <c r="I407" t="inlineStr">
         <is>
           <t>كتيبة حطين</t>
@@ -28260,13 +28228,11 @@
         </is>
       </c>
       <c r="E408" s="1" t="inlineStr"/>
-      <c r="F408" t="inlineStr"/>
       <c r="G408" t="inlineStr">
         <is>
           <t>قائسد مجموعة</t>
         </is>
       </c>
-      <c r="H408" t="inlineStr"/>
       <c r="I408" t="inlineStr">
         <is>
           <t>كتيبة القدس</t>
@@ -28328,13 +28294,11 @@
         </is>
       </c>
       <c r="E409" s="1" t="inlineStr"/>
-      <c r="F409" t="inlineStr"/>
       <c r="G409" t="inlineStr">
         <is>
           <t>قائسد فصيل</t>
         </is>
       </c>
-      <c r="H409" t="inlineStr"/>
       <c r="I409" t="inlineStr">
         <is>
           <t>كتيبة القدس</t>
@@ -28400,13 +28364,11 @@
           <t>2024-03-29</t>
         </is>
       </c>
-      <c r="F410" t="inlineStr"/>
       <c r="G410" t="inlineStr">
         <is>
           <t>مجاهد _ قسامي</t>
         </is>
       </c>
-      <c r="H410" t="inlineStr"/>
       <c r="I410" t="inlineStr">
         <is>
           <t>كتيبة الصحابي أسد الله حمزة</t>
@@ -28472,13 +28434,11 @@
           <t>2024-09-19</t>
         </is>
       </c>
-      <c r="F411" t="inlineStr"/>
       <c r="G411" t="inlineStr">
         <is>
           <t>مجاهد قسا م</t>
         </is>
       </c>
-      <c r="H411" t="inlineStr"/>
       <c r="I411" t="inlineStr">
         <is>
           <t>كتيبة الصحابي أسامة بن زيد</t>
@@ -28544,13 +28504,11 @@
           <t>2023-10-19</t>
         </is>
       </c>
-      <c r="F412" t="inlineStr"/>
       <c r="G412" t="inlineStr">
         <is>
           <t>قائد فصيل</t>
         </is>
       </c>
-      <c r="H412" t="inlineStr"/>
       <c r="I412" t="inlineStr">
         <is>
           <t>كتيبة الشهيد محمد أبو شمالة</t>
@@ -28616,13 +28574,11 @@
           <t>2024-06-28</t>
         </is>
       </c>
-      <c r="F413" t="inlineStr"/>
       <c r="G413" t="inlineStr">
         <is>
           <t>مجاهد قسا م</t>
         </is>
       </c>
-      <c r="H413" t="inlineStr"/>
       <c r="I413" t="inlineStr">
         <is>
           <t>كتيبة الشهيد محمد أبو حرب</t>
@@ -28688,13 +28644,11 @@
           <t>2025-09-09</t>
         </is>
       </c>
-      <c r="F414" t="inlineStr"/>
       <c r="G414" t="inlineStr">
         <is>
           <t>قائد فصيل</t>
         </is>
       </c>
-      <c r="H414" t="inlineStr"/>
       <c r="I414" t="inlineStr">
         <is>
           <t>كتيبة الشهيد محمد الشمالي</t>
@@ -28760,13 +28714,11 @@
           <t>2024-06-09</t>
         </is>
       </c>
-      <c r="F415" t="inlineStr"/>
       <c r="G415" t="inlineStr">
         <is>
           <t>قائد فصيل</t>
         </is>
       </c>
-      <c r="H415" t="inlineStr"/>
       <c r="I415" t="inlineStr">
         <is>
           <t>كتيبة الشهيد رائد العطار</t>
@@ -28832,13 +28784,11 @@
           <t>2023-10-29</t>
         </is>
       </c>
-      <c r="F416" t="inlineStr"/>
       <c r="G416" t="inlineStr">
         <is>
           <t>مجاهد قسا مر</t>
         </is>
       </c>
-      <c r="H416" t="inlineStr"/>
       <c r="I416" t="inlineStr">
         <is>
           <t>كتيبة المدفعية</t>
@@ -28904,13 +28854,11 @@
           <t>2024-05-29</t>
         </is>
       </c>
-      <c r="F417" t="inlineStr"/>
       <c r="G417" t="inlineStr">
         <is>
           <t>قائد فصيل</t>
         </is>
       </c>
-      <c r="H417" t="inlineStr"/>
       <c r="I417" t="inlineStr">
         <is>
           <t>كتيبة الشهيد محمد أبو شمالة</t>
@@ -28976,14 +28924,11 @@
           <t>2023-11-23</t>
         </is>
       </c>
-      <c r="F418" t="inlineStr"/>
       <c r="G418" t="inlineStr">
         <is>
           <t>قائسد سريسة</t>
         </is>
       </c>
-      <c r="H418" t="inlineStr"/>
-      <c r="I418" t="inlineStr"/>
       <c r="J418" t="inlineStr">
         <is>
           <t>لواء رفح</t>
@@ -29044,13 +28989,11 @@
           <t>2024-07-14</t>
         </is>
       </c>
-      <c r="F419" t="inlineStr"/>
       <c r="G419" t="inlineStr">
         <is>
           <t>مجاهد قسا مي</t>
         </is>
       </c>
-      <c r="H419" t="inlineStr"/>
       <c r="I419" t="inlineStr">
         <is>
           <t>كتيبة الشهيد محمد أبو شمالة</t>
@@ -29116,13 +29059,11 @@
           <t>2023-10-13</t>
         </is>
       </c>
-      <c r="F420" t="inlineStr"/>
       <c r="G420" t="inlineStr">
         <is>
           <t>نائب قائد فصيل</t>
         </is>
       </c>
-      <c r="H420" t="inlineStr"/>
       <c r="I420" t="inlineStr">
         <is>
           <t>كتيبة الشهيد عبد الرؤوف نبهان</t>
@@ -29188,13 +29129,11 @@
           <t>2023-10-09</t>
         </is>
       </c>
-      <c r="F421" t="inlineStr"/>
       <c r="G421" t="inlineStr">
         <is>
           <t>قائد فصيل</t>
         </is>
       </c>
-      <c r="H421" t="inlineStr"/>
       <c r="I421" t="inlineStr">
         <is>
           <t>كتيبة الشهيد فوزي أبو القرع</t>
@@ -29260,13 +29199,11 @@
           <t>2024-11-19</t>
         </is>
       </c>
-      <c r="F422" t="inlineStr"/>
       <c r="G422" t="inlineStr">
         <is>
           <t>قائسد سرية</t>
         </is>
       </c>
-      <c r="H422" t="inlineStr"/>
       <c r="I422" t="inlineStr">
         <is>
           <t>كتيبة بيت لاهيا</t>
@@ -29332,13 +29269,11 @@
           <t>2023-10-10</t>
         </is>
       </c>
-      <c r="F423" t="inlineStr"/>
       <c r="G423" t="inlineStr">
         <is>
           <t>نائب قائد فصيل</t>
         </is>
       </c>
-      <c r="H423" t="inlineStr"/>
       <c r="I423" t="inlineStr">
         <is>
           <t>كتيبة الشهيد نضال ناصر</t>
@@ -29404,13 +29339,11 @@
           <t>2025-06-20</t>
         </is>
       </c>
-      <c r="F424" t="inlineStr"/>
       <c r="G424" t="inlineStr">
         <is>
           <t>قائد سرية</t>
         </is>
       </c>
-      <c r="H424" t="inlineStr"/>
       <c r="I424" t="inlineStr">
         <is>
           <t>كتيبة الشهيد عماد عقل</t>
@@ -29476,13 +29409,11 @@
           <t>2023</t>
         </is>
       </c>
-      <c r="F425" t="inlineStr"/>
       <c r="G425" t="inlineStr">
         <is>
           <t>قائد مجموعة</t>
         </is>
       </c>
-      <c r="H425" t="inlineStr"/>
       <c r="I425" t="inlineStr">
         <is>
           <t>كتيبة الشهيد عماد عقل</t>
@@ -29544,13 +29475,11 @@
           <t>2024-05-24</t>
         </is>
       </c>
-      <c r="F426" t="inlineStr"/>
       <c r="G426" t="inlineStr">
         <is>
           <t>قائسد فصيل</t>
         </is>
       </c>
-      <c r="H426" t="inlineStr"/>
       <c r="I426" t="inlineStr">
         <is>
           <t>كتيبة الشهيد سهيل زيادة</t>
@@ -29587,6 +29516,146 @@
         </is>
       </c>
       <c r="P426" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="n">
+        <v>922</v>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>بلال محمد جودة</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>بلال محمد جوده</t>
+        </is>
+      </c>
+      <c r="D427" s="1" t="inlineStr">
+        <is>
+          <t>1987-02-15</t>
+        </is>
+      </c>
+      <c r="E427" s="1" t="inlineStr">
+        <is>
+          <t>2024-11-05</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>قائد سرية</t>
+        </is>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>كتيبة الشهيد عبد الرؤوف نبهان</t>
+        </is>
+      </c>
+      <c r="J427" t="inlineStr">
+        <is>
+          <t>لواء الشمال</t>
+        </is>
+      </c>
+      <c r="K427" t="inlineStr">
+        <is>
+          <t>data/photos\922.jpg</t>
+        </is>
+      </c>
+      <c r="L427" t="inlineStr">
+        <is>
+          <t>data/frames\922_28.jpg;data/frames\922_30.jpg;data/frames\922_32.jpg</t>
+        </is>
+      </c>
+      <c r="M427" t="inlineStr">
+        <is>
+          <t>2026-05-16 20:01</t>
+        </is>
+      </c>
+      <c r="N427" t="inlineStr">
+        <is>
+          <t>https://t.me/AqmarTofan/922</t>
+        </is>
+      </c>
+      <c r="O427" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="P427" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="n">
+        <v>924</v>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>خالد علي عبد الرحمن</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>خالد علي عبد الرحمن</t>
+        </is>
+      </c>
+      <c r="D428" s="1" t="inlineStr">
+        <is>
+          <t>1962-01-08</t>
+        </is>
+      </c>
+      <c r="E428" s="1" t="inlineStr">
+        <is>
+          <t>2023-11-29</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>قائد فصيل</t>
+        </is>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>كتيبة حطين</t>
+        </is>
+      </c>
+      <c r="J428" t="inlineStr">
+        <is>
+          <t>لواء الوسطى</t>
+        </is>
+      </c>
+      <c r="K428" t="inlineStr">
+        <is>
+          <t>data/photos\924.jpg</t>
+        </is>
+      </c>
+      <c r="L428" t="inlineStr">
+        <is>
+          <t>data/frames\924_28.jpg;data/frames\924_30.jpg;data/frames\924_32.jpg</t>
+        </is>
+      </c>
+      <c r="M428" t="inlineStr">
+        <is>
+          <t>2026-05-17 07:03</t>
+        </is>
+      </c>
+      <c r="N428" t="inlineStr">
+        <is>
+          <t>https://t.me/AqmarTofan/924</t>
+        </is>
+      </c>
+      <c r="O428" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+      <c r="P428" t="inlineStr">
         <is>
           <t>unique</t>
         </is>

</xml_diff>